<commit_message>
reports: add verified GC emails / sub-intake channels to permit call sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0151ZApF1udXvgWuNKWDLg8z
</commit_message>
<xml_diff>
--- a/tender-system/reports/permit-GC-crews-2026-09-10.xlsx
+++ b/tender-system/reports/permit-GC-crews-2026-09-10.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q368"/>
+  <dimension ref="A1:R368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -451,6 +451,7 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="22" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -539,6 +540,11 @@
           <t>Следующий шаг</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Вход для субов / заметки (веб)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -732,6 +738,11 @@
       </c>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>https://ryconinc.com/sub-contractors/ (форма + MSA)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -791,6 +802,11 @@
       </c>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>buildwithnovacm.com/contact/ форма; Coral Gables, 2–10 чел.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -865,7 +881,11 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>info@hawkinsnet.com</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>DRAFTED</t>
@@ -908,6 +928,11 @@
       </c>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>hawkinsplanroom.com; Boca (561) 314-6730</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1046,7 +1071,11 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>info@firstflorida.com</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -1087,6 +1116,11 @@
       </c>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>firstflorida.com/become-a-trade-partner (BuildingConnected)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1145,6 +1179,11 @@
       </c>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>форма rubioconstruction.com/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1202,6 +1241,11 @@
       </c>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>альт. (954) 541-5172; Jonathan Warren</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1682,7 +1726,11 @@
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>AFigueroa@MadisonGC.com (не подтверждён)</t>
+        </is>
+      </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -1725,6 +1773,11 @@
       </c>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>madisongc.com форма</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1741,7 +1794,11 @@
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>info@excelsf.com</t>
+        </is>
+      </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -1782,6 +1839,11 @@
       </c>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Davie</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1840,6 +1902,11 @@
       </c>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>альт. (954) 668-8623; Richard Leger</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1897,6 +1964,11 @@
       </c>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>альт. (305) 778-5961; Jose Sbarra</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1913,7 +1985,11 @@
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>phuntington@butters.com; jcusmano@butters.com; jleal@butters.com; info@butters.com</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -1955,6 +2031,11 @@
       </c>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>butters.com/project-bidding/ — Peter Huntington 954-312-2404</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2076,6 +2157,11 @@
       </c>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>juneaucc.com/trade-partners/ → Procore; Coral Gables (305) 438-7666</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2149,7 +2235,11 @@
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>office@ncgflorida.com</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -2192,6 +2282,11 @@
       </c>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>nielconstructiongroup.com/vendors (W-9 + COI)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2323,7 +2418,11 @@
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>info@buildalcon.com</t>
+        </is>
+      </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>DRAFTED</t>
@@ -2366,6 +2465,11 @@
       </c>
       <c r="P32" s="2" t="inlineStr"/>
       <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>альт. 786-349-3070; Charlie Alvarez</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2838,6 +2942,11 @@
       </c>
       <c r="P40" s="2" t="inlineStr"/>
       <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>camcongroup.com/become-a-subcontractor/; альт. (305) 447-2999</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2854,7 +2963,11 @@
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>info@alartechinc.com</t>
+        </is>
+      </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -2897,6 +3010,11 @@
       </c>
       <c r="P41" s="2" t="inlineStr"/>
       <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>спросить Alex</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2976,7 +3094,11 @@
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>contact@skycongroup.com</t>
+        </is>
+      </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -3018,6 +3140,11 @@
       </c>
       <c r="P43" s="2" t="inlineStr"/>
       <c r="Q43" s="2" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>commercial interiors, 200+ проектов</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -3272,7 +3399,11 @@
           <t>(305) 443-5808</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Info@usconstructioncorp.com</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
           <t>DRAFTED</t>
@@ -3315,6 +3446,11 @@
       </c>
       <c r="P48" s="2" t="inlineStr"/>
       <c r="Q48" s="2" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>usconstructioncorp.com/become-subcontractor (COI $1M, W-9, EMR, refs)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -3331,7 +3467,11 @@
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>info@kennedycompanies.com</t>
+        </is>
+      </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
           <t>NEW</t>
@@ -3372,6 +3512,11 @@
       </c>
       <c r="P49" s="2" t="inlineStr"/>
       <c r="Q49" s="2" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>WPB</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -3450,7 +3595,11 @@
           <t>(305) 649-7509</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>info@yagarconstruction.com</t>
+        </is>
+      </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
           <t>DRAFTED</t>
@@ -3493,6 +3642,11 @@
       </c>
       <c r="P51" s="2" t="inlineStr"/>
       <c r="Q51" s="2" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Carlos Garcia, семейная с 1968</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">

</xml_diff>